<commit_message>
Add scenario (multi-step) test support and pre-flight validation
Introduce a Scenario Name column so consecutive rows can be uploaded
and compared as the steps of one Applitools test instead of one test
per row, matching how the Applitools Figma plugin itself uploads a
multi-frame scenario (confirmed via HAR inspection). Add FigmaValidation
to catch missing fields, non-contiguous scenarios, conflicting
scenario metadata, and (for Android) missing screen flows before any
real work starts. Rework Baseline, UploadFromFigma, BajajFinservWebTest,
and BajajFinservAndroidTest to operate on row groups instead of single
rows, with a standalone row modeled as a group of one.
</commit_message>
<xml_diff>
--- a/figma-visual-testing/templates/figma_visual_tests_template.xlsx
+++ b/figma-visual-testing/templates/figma_visual_tests_template.xlsx
@@ -423,25 +423,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:Q8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="65" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
     <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="45" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="30" customWidth="1" min="14" max="14"/>
-    <col width="45" customWidth="1" min="15" max="15"/>
-    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="45" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="30" customWidth="1" min="15" max="15"/>
+    <col width="45" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -462,65 +463,70 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Scenario Name</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Baseline Env Name</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Viewport</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Scale</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Format</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Skip</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>App Name</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Baseline Batch URL</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Error Message</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Locator</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Comparison Batch URL</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Validation Status</t>
         </is>
@@ -555,6 +561,7 @@
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -572,43 +579,44 @@
           <t>https://uat.example.com/cards</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
         <is>
           <t>cards-component</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>cards-component-custom-baseline</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>1280x1024</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>png</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr">
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr">
         <is>
           <t>#main-content &gt; div.cards-section</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -626,12 +634,12 @@
           <t>Home Screen</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
         <is>
           <t>android-home-screen</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
@@ -643,11 +651,12 @@
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>https://www.figma.com/design/abc123XYZ/My-Project?node-id=99-111</t>
+          <t>https://www.figma.com/design/abc123XYZ/My-Project?node-id=20-1</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -657,19 +666,23 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://uat.example.com/not-ready-yet</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
+          <t>https://uat.example.com/home</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>applitools-web-flow</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Applitools Home</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Skip</t>
-        </is>
-      </c>
+      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
@@ -677,6 +690,120 @@
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/abc123XYZ/My-Project?node-id=20-2</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://uat.example.com/whats-new</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>applitools-web-flow</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Whats New</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/abc123XYZ/My-Project?node-id=20-3</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://uat.example.com/integrate</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>applitools-web-flow</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Integrate</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/abc123XYZ/My-Project?node-id=99-111</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://uat.example.com/not-ready-yet</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Skip</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Rework Android compareWithFigma around a shared scenario registry
Make Scenario Name mandatory for every Android/iOS row, since even a
single mobile screen can need bespoke login/navigation - there's no
generic per-screen runner the way web has. Introduce
AndroidScenarioRegistry so scenario implementations can live in any
class file and be discovered by name, ScenarioFlow as the bespoke
test-procedure contract, and CompareAndroidWithFigma as the one
runner for every app. BajajFinservAndroidTest becomes a pure scenario
provider instead of owning its own TestNG lifecycle.
</commit_message>
<xml_diff>
--- a/figma-visual-testing/templates/figma_visual_tests_template.xlsx
+++ b/figma-visual-testing/templates/figma_visual_tests_template.xlsx
@@ -634,7 +634,11 @@
           <t>Home Screen</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>android-home-screen</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>android-home-screen</t>

</xml_diff>

<commit_message>
Add cleanFigmaExcel Gradle task; reorder template columns to match
</commit_message>
<xml_diff>
--- a/figma-visual-testing/templates/figma_visual_tests_template.xlsx
+++ b/figma-visual-testing/templates/figma_visual_tests_template.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,22 +25,13 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DDEBF7"/>
-        <bgColor rgb="00DDEBF7"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -55,9 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,108 +415,89 @@
   </sheetPr>
   <dimension ref="A1:Q8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="65" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="45" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="30" customWidth="1" min="15" max="15"/>
-    <col width="45" customWidth="1" min="16" max="16"/>
-    <col width="16" customWidth="1" min="17" max="17"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Figma URL</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>App URL / Screen Name</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Scenario Name</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Baseline Env Name</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Viewport</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Scale</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Format</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Skip</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Locator</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
         <is>
           <t>App Name</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Baseline Batch URL</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Error Message</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Locator</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Comparison Batch URL</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Validation Status</t>
         </is>
@@ -548,20 +519,6 @@
           <t>https://uat.example.com/homepage</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -579,7 +536,6 @@
           <t>https://uat.example.com/cards</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>cards-component</t>
@@ -605,18 +561,11 @@
           <t>png</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>#main-content &gt; div.cards-section</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -644,18 +593,6 @@
           <t>android-home-screen</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -683,18 +620,6 @@
           <t>Applitools Home</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -722,18 +647,6 @@
           <t>Whats New</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -761,18 +674,6 @@
           <t>Integrate</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -790,24 +691,11 @@
           <t>https://uat.example.com/not-ready-yet</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
           <t>Skip</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>